<commit_message>
feat: update test cases to use single check_point value and replace spreadsheet files
</commit_message>
<xml_diff>
--- a/tests/files/planilhas/planilha_Form-test-example-with-images_error_modelo.xlsx
+++ b/tests/files/planilhas/planilha_Form-test-example-with-images_error_modelo.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="29">
   <si>
     <t xml:space="preserve">uc</t>
   </si>
@@ -83,12 +83,6 @@
   </si>
   <si>
     <t xml:space="preserve">dezoito</t>
-  </si>
-  <si>
-    <t xml:space="preserve">vinte e oito</t>
-  </si>
-  <si>
-    <t xml:space="preserve">trinta e oito</t>
   </si>
   <si>
     <t xml:space="preserve">Floresta Nacional de Brasília</t>
@@ -404,7 +398,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H1048576"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="36"/>
@@ -487,69 +481,45 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>24</v>
+      </c>
       <c r="E4" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>28</v>
+      </c>
       <c r="E5" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E7" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E8" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E10" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E11" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>